<commit_message>
docs(v2.8.0): add project analysis report and assessment documents
- Add comprehensive v2.8.0 project analysis report (docs/report/)
- Add project analysis guide with workflow and tool instructions
- Add v2.8.0 version-specific analysis report (docs/governance/reports/)
- Update Minimax usage analysis with latest CSV data (04-24)
- Update trend chart scripts and generated charts
- Update 项目分析报告.md with latest data through 04-22

Key findings:
- v2.8.0: 81 PRs in 2 days, distributed features (GTID/semi-sync/read-write split)
- Minimax: 4.37B tokens/day (last 2 weeks), +44.3% vs prior 2 weeks
- TPC-H SF=1: 22/22 queries pass, total ~4.2s (v2.7.0)
- Sysbench OLTP: 55K TPS point select, 22K TPS insert
- Documentation PRs at 31.7% - project entering maturity phase
</commit_message>
<xml_diff>
--- a/scripts/usage/minimax_usage_summary.xlsx
+++ b/scripts/usage/minimax_usage_summary.xlsx
@@ -10,13 +10,22 @@
     <sheet name="每日汇总" sheetId="1" r:id="rId1"/>
     <sheet name="每周汇总" sheetId="2" r:id="rId2"/>
     <sheet name="每月汇总" sheetId="3" r:id="rId3"/>
+    <sheet name="最近2周" sheetId="4" r:id="rId4"/>
+    <sheet name="模型分布" sheetId="5" r:id="rId5"/>
+    <sheet name="接口分布" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="17">
+  <si>
+    <t>输入消费数</t>
+  </si>
+  <si>
+    <t>输出消费数</t>
+  </si>
   <si>
     <t>总消费数</t>
   </si>
@@ -25,6 +34,42 @@
   </si>
   <si>
     <t>日期</t>
+  </si>
+  <si>
+    <t>消费模型</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.7-highspeed</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.1</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.7</t>
+  </si>
+  <si>
+    <t>coding-plan-search</t>
+  </si>
+  <si>
+    <t>subscribe</t>
+  </si>
+  <si>
+    <t>消费接口</t>
+  </si>
+  <si>
+    <t>cache-read(Text API)</t>
+  </si>
+  <si>
+    <t>chatcompletion-v2(Text API)</t>
+  </si>
+  <si>
+    <t>cache-create(Text API)</t>
+  </si>
+  <si>
+    <t>code_plan_resource_package</t>
+  </si>
+  <si>
+    <t>code_plan_purchase</t>
   </si>
 </sst>
 </file>
@@ -360,12 +405,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -373,742 +418,1201 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>46055</v>
       </c>
       <c r="B2">
+        <v>44109875</v>
+      </c>
+      <c r="C2">
+        <v>193229</v>
+      </c>
+      <c r="D2">
         <v>44303104</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>46056</v>
       </c>
       <c r="B3">
+        <v>24346019</v>
+      </c>
+      <c r="C3">
+        <v>69189</v>
+      </c>
+      <c r="D3">
         <v>24415208</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>46058</v>
       </c>
       <c r="B4">
+        <v>68473</v>
+      </c>
+      <c r="C4">
+        <v>723</v>
+      </c>
+      <c r="D4">
         <v>69196</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>46062</v>
       </c>
       <c r="B5">
+        <v>223019</v>
+      </c>
+      <c r="C5">
+        <v>3189</v>
+      </c>
+      <c r="D5">
         <v>226208</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>46064</v>
       </c>
       <c r="B6">
+        <v>1625031</v>
+      </c>
+      <c r="C6">
+        <v>50080</v>
+      </c>
+      <c r="D6">
         <v>1675111</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>46065</v>
       </c>
       <c r="B7">
+        <v>10098026</v>
+      </c>
+      <c r="C7">
+        <v>80296</v>
+      </c>
+      <c r="D7">
         <v>10178322</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>46066</v>
       </c>
       <c r="B8">
+        <v>195262132</v>
+      </c>
+      <c r="C8">
+        <v>1014368</v>
+      </c>
+      <c r="D8">
         <v>196276500</v>
       </c>
-      <c r="C8">
+      <c r="E8">
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>46067</v>
       </c>
       <c r="B9">
+        <v>118553679</v>
+      </c>
+      <c r="C9">
+        <v>540118</v>
+      </c>
+      <c r="D9">
         <v>119093797</v>
       </c>
-      <c r="C9">
+      <c r="E9">
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>46068</v>
       </c>
       <c r="B10">
+        <v>107894789</v>
+      </c>
+      <c r="C10">
+        <v>740115</v>
+      </c>
+      <c r="D10">
         <v>108634904</v>
       </c>
-      <c r="C10">
+      <c r="E10">
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1">
         <v>46069</v>
       </c>
       <c r="B11">
+        <v>140301200</v>
+      </c>
+      <c r="C11">
+        <v>1178444</v>
+      </c>
+      <c r="D11">
         <v>141479644</v>
       </c>
-      <c r="C11">
+      <c r="E11">
         <v>144</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:5">
       <c r="A12" s="1">
         <v>46070</v>
       </c>
       <c r="B12">
+        <v>170014054</v>
+      </c>
+      <c r="C12">
+        <v>606139</v>
+      </c>
+      <c r="D12">
         <v>170620193</v>
       </c>
-      <c r="C12">
+      <c r="E12">
         <v>144</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:5">
       <c r="A13" s="1">
         <v>46071</v>
       </c>
       <c r="B13">
+        <v>121481164</v>
+      </c>
+      <c r="C13">
+        <v>452181</v>
+      </c>
+      <c r="D13">
         <v>121933345</v>
       </c>
-      <c r="C13">
+      <c r="E13">
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:5">
       <c r="A14" s="1">
         <v>46072</v>
       </c>
       <c r="B14">
+        <v>39782200</v>
+      </c>
+      <c r="C14">
+        <v>294745</v>
+      </c>
+      <c r="D14">
         <v>40076945</v>
       </c>
-      <c r="C14">
+      <c r="E14">
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:5">
       <c r="A15" s="1">
         <v>46073</v>
       </c>
       <c r="B15">
+        <v>259713471</v>
+      </c>
+      <c r="C15">
+        <v>1000667</v>
+      </c>
+      <c r="D15">
         <v>260714138</v>
       </c>
-      <c r="C15">
+      <c r="E15">
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:5">
       <c r="A16" s="1">
         <v>46074</v>
       </c>
       <c r="B16">
+        <v>66491505</v>
+      </c>
+      <c r="C16">
+        <v>247164</v>
+      </c>
+      <c r="D16">
         <v>66738669</v>
       </c>
-      <c r="C16">
+      <c r="E16">
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:5">
       <c r="A17" s="1">
         <v>46075</v>
       </c>
       <c r="B17">
+        <v>5513297</v>
+      </c>
+      <c r="C17">
+        <v>42902</v>
+      </c>
+      <c r="D17">
         <v>5556199</v>
       </c>
-      <c r="C17">
+      <c r="E17">
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:5">
       <c r="A18" s="1">
         <v>46076</v>
       </c>
       <c r="B18">
+        <v>1136491</v>
+      </c>
+      <c r="C18">
+        <v>4019</v>
+      </c>
+      <c r="D18">
         <v>1140510</v>
       </c>
-      <c r="C18">
+      <c r="E18">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:5">
       <c r="A19" s="1">
         <v>46077</v>
       </c>
       <c r="B19">
+        <v>2606410</v>
+      </c>
+      <c r="C19">
+        <v>26537</v>
+      </c>
+      <c r="D19">
         <v>2632947</v>
       </c>
-      <c r="C19">
+      <c r="E19">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:5">
       <c r="A20" s="1">
         <v>46081</v>
       </c>
       <c r="B20">
+        <v>3890043</v>
+      </c>
+      <c r="C20">
+        <v>24291</v>
+      </c>
+      <c r="D20">
         <v>3914334</v>
       </c>
-      <c r="C20">
+      <c r="E20">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:5">
       <c r="A21" s="1">
         <v>46082</v>
       </c>
       <c r="B21">
+        <v>76442533</v>
+      </c>
+      <c r="C21">
+        <v>111170</v>
+      </c>
+      <c r="D21">
         <v>76553703</v>
       </c>
-      <c r="C21">
+      <c r="E21">
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:5">
       <c r="A22" s="1">
         <v>46083</v>
       </c>
       <c r="B22">
+        <v>10806084</v>
+      </c>
+      <c r="C22">
+        <v>30789</v>
+      </c>
+      <c r="D22">
         <v>10836873</v>
       </c>
-      <c r="C22">
+      <c r="E22">
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:5">
       <c r="A23" s="1">
         <v>46084</v>
       </c>
       <c r="B23">
+        <v>260321813</v>
+      </c>
+      <c r="C23">
+        <v>949069</v>
+      </c>
+      <c r="D23">
         <v>261270882</v>
       </c>
-      <c r="C23">
+      <c r="E23">
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:5">
       <c r="A24" s="1">
         <v>46085</v>
       </c>
       <c r="B24">
+        <v>57609431</v>
+      </c>
+      <c r="C24">
+        <v>169857</v>
+      </c>
+      <c r="D24">
         <v>57779288</v>
       </c>
-      <c r="C24">
+      <c r="E24">
         <v>88</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:5">
       <c r="A25" s="1">
         <v>46086</v>
       </c>
       <c r="B25">
+        <v>432659759</v>
+      </c>
+      <c r="C25">
+        <v>1367934</v>
+      </c>
+      <c r="D25">
         <v>434027693</v>
       </c>
-      <c r="C25">
+      <c r="E25">
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:5">
       <c r="A26" s="1">
         <v>46087</v>
       </c>
       <c r="B26">
+        <v>69824048</v>
+      </c>
+      <c r="C26">
+        <v>126022</v>
+      </c>
+      <c r="D26">
         <v>69950070</v>
       </c>
-      <c r="C26">
+      <c r="E26">
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:5">
       <c r="A27" s="1">
         <v>46088</v>
       </c>
       <c r="B27">
+        <v>123888083</v>
+      </c>
+      <c r="C27">
+        <v>526914</v>
+      </c>
+      <c r="D27">
         <v>124414997</v>
       </c>
-      <c r="C27">
+      <c r="E27">
         <v>96</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:5">
       <c r="A28" s="1">
         <v>46089</v>
       </c>
       <c r="B28">
+        <v>94927345</v>
+      </c>
+      <c r="C28">
+        <v>206477</v>
+      </c>
+      <c r="D28">
         <v>95133822</v>
       </c>
-      <c r="C28">
+      <c r="E28">
         <v>104</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:5">
       <c r="A29" s="1">
         <v>46090</v>
       </c>
       <c r="B29">
+        <v>40431889</v>
+      </c>
+      <c r="C29">
+        <v>169386</v>
+      </c>
+      <c r="D29">
         <v>40601275</v>
       </c>
-      <c r="C29">
+      <c r="E29">
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:5">
       <c r="A30" s="1">
         <v>46091</v>
       </c>
       <c r="B30">
+        <v>17773567</v>
+      </c>
+      <c r="C30">
+        <v>99491</v>
+      </c>
+      <c r="D30">
         <v>17873058</v>
       </c>
-      <c r="C30">
+      <c r="E30">
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:5">
       <c r="A31" s="1">
         <v>46092</v>
       </c>
       <c r="B31">
+        <v>217635219</v>
+      </c>
+      <c r="C31">
+        <v>736629</v>
+      </c>
+      <c r="D31">
         <v>218371848</v>
       </c>
-      <c r="C31">
+      <c r="E31">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:5">
       <c r="A32" s="1">
         <v>46093</v>
       </c>
       <c r="B32">
+        <v>65692490</v>
+      </c>
+      <c r="C32">
+        <v>208372</v>
+      </c>
+      <c r="D32">
         <v>65900862</v>
       </c>
-      <c r="C32">
+      <c r="E32">
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:5">
       <c r="A33" s="1">
         <v>46094</v>
       </c>
       <c r="B33">
+        <v>150670082</v>
+      </c>
+      <c r="C33">
+        <v>508790</v>
+      </c>
+      <c r="D33">
         <v>151178872</v>
       </c>
-      <c r="C33">
+      <c r="E33">
         <v>87</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:5">
       <c r="A34" s="1">
         <v>46095</v>
       </c>
       <c r="B34">
+        <v>131208124</v>
+      </c>
+      <c r="C34">
+        <v>318055</v>
+      </c>
+      <c r="D34">
         <v>131526179</v>
       </c>
-      <c r="C34">
+      <c r="E34">
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:5">
       <c r="A35" s="1">
         <v>46096</v>
       </c>
       <c r="B35">
+        <v>229056688</v>
+      </c>
+      <c r="C35">
+        <v>539232</v>
+      </c>
+      <c r="D35">
         <v>229595920</v>
       </c>
-      <c r="C35">
+      <c r="E35">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:5">
       <c r="A36" s="1">
         <v>46097</v>
       </c>
       <c r="B36">
+        <v>143019798</v>
+      </c>
+      <c r="C36">
+        <v>333861</v>
+      </c>
+      <c r="D36">
         <v>143353659</v>
       </c>
-      <c r="C36">
+      <c r="E36">
         <v>93</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:5">
       <c r="A37" s="1">
         <v>46098</v>
       </c>
       <c r="B37">
+        <v>11928233</v>
+      </c>
+      <c r="C37">
+        <v>51737</v>
+      </c>
+      <c r="D37">
         <v>11979970</v>
       </c>
-      <c r="C37">
+      <c r="E37">
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:5">
       <c r="A38" s="1">
         <v>46099</v>
       </c>
       <c r="B38">
+        <v>399975698</v>
+      </c>
+      <c r="C38">
+        <v>772414</v>
+      </c>
+      <c r="D38">
         <v>400748112</v>
       </c>
-      <c r="C38">
+      <c r="E38">
         <v>96</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:5">
       <c r="A39" s="1">
         <v>46100</v>
       </c>
       <c r="B39">
+        <v>609350469</v>
+      </c>
+      <c r="C39">
+        <v>1236187</v>
+      </c>
+      <c r="D39">
         <v>610586656</v>
       </c>
-      <c r="C39">
+      <c r="E39">
         <v>106</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:5">
       <c r="A40" s="1">
         <v>46101</v>
       </c>
       <c r="B40">
+        <v>256702111</v>
+      </c>
+      <c r="C40">
+        <v>469772</v>
+      </c>
+      <c r="D40">
         <v>257171883</v>
       </c>
-      <c r="C40">
+      <c r="E40">
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:5">
       <c r="A41" s="1">
         <v>46102</v>
       </c>
       <c r="B41">
+        <v>395205934</v>
+      </c>
+      <c r="C41">
+        <v>970120</v>
+      </c>
+      <c r="D41">
         <v>396176054</v>
       </c>
-      <c r="C41">
+      <c r="E41">
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:5">
       <c r="A42" s="1">
         <v>46103</v>
       </c>
       <c r="B42">
+        <v>24127943</v>
+      </c>
+      <c r="C42">
+        <v>86128</v>
+      </c>
+      <c r="D42">
         <v>24214071</v>
       </c>
-      <c r="C42">
+      <c r="E42">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:5">
       <c r="A43" s="1">
         <v>46104</v>
       </c>
       <c r="B43">
+        <v>83691704</v>
+      </c>
+      <c r="C43">
+        <v>214302</v>
+      </c>
+      <c r="D43">
         <v>83906006</v>
       </c>
-      <c r="C43">
+      <c r="E43">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:5">
       <c r="A44" s="1">
         <v>46105</v>
       </c>
       <c r="B44">
+        <v>69644470</v>
+      </c>
+      <c r="C44">
+        <v>207355</v>
+      </c>
+      <c r="D44">
         <v>69851825</v>
       </c>
-      <c r="C44">
+      <c r="E44">
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:5">
       <c r="A45" s="1">
         <v>46106</v>
       </c>
       <c r="B45">
+        <v>61827053</v>
+      </c>
+      <c r="C45">
+        <v>125764</v>
+      </c>
+      <c r="D45">
         <v>61952817</v>
       </c>
-      <c r="C45">
+      <c r="E45">
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:5">
       <c r="A46" s="1">
         <v>46107</v>
       </c>
       <c r="B46">
+        <v>801621176</v>
+      </c>
+      <c r="C46">
+        <v>3000001</v>
+      </c>
+      <c r="D46">
         <v>804621177</v>
       </c>
-      <c r="C46">
+      <c r="E46">
         <v>121</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:5">
       <c r="A47" s="1">
         <v>46108</v>
       </c>
       <c r="B47">
+        <v>410302751</v>
+      </c>
+      <c r="C47">
+        <v>1260959</v>
+      </c>
+      <c r="D47">
         <v>411563710</v>
       </c>
-      <c r="C47">
+      <c r="E47">
         <v>79</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:5">
       <c r="A48" s="1">
         <v>46109</v>
       </c>
       <c r="B48">
+        <v>669961980</v>
+      </c>
+      <c r="C48">
+        <v>2390124</v>
+      </c>
+      <c r="D48">
         <v>672352104</v>
       </c>
-      <c r="C48">
+      <c r="E48">
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:5">
       <c r="A49" s="1">
         <v>46110</v>
       </c>
       <c r="B49">
+        <v>781214642</v>
+      </c>
+      <c r="C49">
+        <v>2860496</v>
+      </c>
+      <c r="D49">
         <v>784075138</v>
       </c>
-      <c r="C49">
+      <c r="E49">
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:5">
       <c r="A50" s="1">
         <v>46111</v>
       </c>
       <c r="B50">
+        <v>228863225</v>
+      </c>
+      <c r="C50">
+        <v>942753</v>
+      </c>
+      <c r="D50">
         <v>229805978</v>
       </c>
-      <c r="C50">
+      <c r="E50">
         <v>80</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:5">
       <c r="A51" s="1">
         <v>46112</v>
       </c>
       <c r="B51">
+        <v>137185545</v>
+      </c>
+      <c r="C51">
+        <v>487997</v>
+      </c>
+      <c r="D51">
         <v>137673542</v>
       </c>
-      <c r="C51">
+      <c r="E51">
         <v>82</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:5">
       <c r="A52" s="1">
         <v>46113</v>
       </c>
       <c r="B52">
+        <v>315751692</v>
+      </c>
+      <c r="C52">
+        <v>1016666</v>
+      </c>
+      <c r="D52">
         <v>316768358</v>
       </c>
-      <c r="C52">
+      <c r="E52">
         <v>87</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:5">
       <c r="A53" s="1">
         <v>46114</v>
       </c>
       <c r="B53">
+        <v>455846463</v>
+      </c>
+      <c r="C53">
+        <v>1163341</v>
+      </c>
+      <c r="D53">
         <v>457009804</v>
       </c>
-      <c r="C53">
+      <c r="E53">
         <v>80</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:5">
       <c r="A54" s="1">
         <v>46115</v>
       </c>
       <c r="B54">
+        <v>173451910</v>
+      </c>
+      <c r="C54">
+        <v>867510</v>
+      </c>
+      <c r="D54">
         <v>174319420</v>
       </c>
-      <c r="C54">
+      <c r="E54">
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:5">
       <c r="A55" s="1">
         <v>46116</v>
       </c>
       <c r="B55">
+        <v>163888833</v>
+      </c>
+      <c r="C55">
+        <v>679765</v>
+      </c>
+      <c r="D55">
         <v>164568598</v>
       </c>
-      <c r="C55">
+      <c r="E55">
         <v>93</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:5">
       <c r="A56" s="1">
         <v>46117</v>
       </c>
       <c r="B56">
+        <v>88121</v>
+      </c>
+      <c r="C56">
+        <v>104</v>
+      </c>
+      <c r="D56">
         <v>88225</v>
       </c>
-      <c r="C56">
+      <c r="E56">
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:5">
       <c r="A57" s="1">
         <v>46119</v>
       </c>
       <c r="B57">
+        <v>52904173</v>
+      </c>
+      <c r="C57">
+        <v>607681</v>
+      </c>
+      <c r="D57">
         <v>53511854</v>
       </c>
-      <c r="C57">
+      <c r="E57">
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:5">
       <c r="A58" s="1">
         <v>46120</v>
       </c>
       <c r="B58">
+        <v>224034425</v>
+      </c>
+      <c r="C58">
+        <v>522473</v>
+      </c>
+      <c r="D58">
         <v>224556898</v>
       </c>
-      <c r="C58">
+      <c r="E58">
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:5">
       <c r="A59" s="1">
         <v>46121</v>
       </c>
       <c r="B59">
+        <v>309706503</v>
+      </c>
+      <c r="C59">
+        <v>874609</v>
+      </c>
+      <c r="D59">
         <v>310581112</v>
       </c>
-      <c r="C59">
+      <c r="E59">
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:5">
       <c r="A60" s="1">
         <v>46122</v>
       </c>
       <c r="B60">
+        <v>116346489</v>
+      </c>
+      <c r="C60">
+        <v>289339</v>
+      </c>
+      <c r="D60">
         <v>116635828</v>
       </c>
-      <c r="C60">
+      <c r="E60">
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:5">
       <c r="A61" s="1">
         <v>46123</v>
       </c>
       <c r="B61">
+        <v>160607016</v>
+      </c>
+      <c r="C61">
+        <v>686187</v>
+      </c>
+      <c r="D61">
         <v>161293203</v>
       </c>
-      <c r="C61">
+      <c r="E61">
         <v>54</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:5">
       <c r="A62" s="1">
         <v>46124</v>
       </c>
       <c r="B62">
+        <v>475094565</v>
+      </c>
+      <c r="C62">
+        <v>1908297</v>
+      </c>
+      <c r="D62">
         <v>477002862</v>
       </c>
-      <c r="C62">
+      <c r="E62">
         <v>82</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:5">
       <c r="A63" s="1">
         <v>46125</v>
       </c>
       <c r="B63">
+        <v>256361479</v>
+      </c>
+      <c r="C63">
+        <v>824687</v>
+      </c>
+      <c r="D63">
         <v>257186166</v>
       </c>
-      <c r="C63">
+      <c r="E63">
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:5">
       <c r="A64" s="1">
         <v>46126</v>
       </c>
       <c r="B64">
+        <v>277328285</v>
+      </c>
+      <c r="C64">
+        <v>875263</v>
+      </c>
+      <c r="D64">
         <v>278203548</v>
       </c>
-      <c r="C64">
+      <c r="E64">
         <v>102</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:5">
       <c r="A65" s="1">
         <v>46127</v>
       </c>
       <c r="B65">
+        <v>204982226</v>
+      </c>
+      <c r="C65">
+        <v>952185</v>
+      </c>
+      <c r="D65">
         <v>205934411</v>
       </c>
-      <c r="C65">
+      <c r="E65">
         <v>69</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:5">
       <c r="A66" s="1">
         <v>46128</v>
       </c>
       <c r="B66">
+        <v>984805312</v>
+      </c>
+      <c r="C66">
+        <v>3225513</v>
+      </c>
+      <c r="D66">
         <v>988030825</v>
       </c>
-      <c r="C66">
+      <c r="E66">
         <v>93</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:5">
       <c r="A67" s="1">
         <v>46129</v>
       </c>
       <c r="B67">
+        <v>481719807</v>
+      </c>
+      <c r="C67">
+        <v>1434059</v>
+      </c>
+      <c r="D67">
         <v>483153866</v>
       </c>
-      <c r="C67">
+      <c r="E67">
         <v>104</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:5">
       <c r="A68" s="1">
         <v>46130</v>
       </c>
       <c r="B68">
+        <v>984655867</v>
+      </c>
+      <c r="C68">
+        <v>4639910</v>
+      </c>
+      <c r="D68">
         <v>989295777</v>
       </c>
-      <c r="C68">
+      <c r="E68">
         <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B69">
+        <v>540208877</v>
+      </c>
+      <c r="C69">
+        <v>2033591</v>
+      </c>
+      <c r="D69">
+        <v>542242468</v>
+      </c>
+      <c r="E69">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B70">
+        <v>164639448</v>
+      </c>
+      <c r="C70">
+        <v>781460</v>
+      </c>
+      <c r="D70">
+        <v>165420908</v>
+      </c>
+      <c r="E70">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B71">
+        <v>578105107</v>
+      </c>
+      <c r="C71">
+        <v>2008594</v>
+      </c>
+      <c r="D71">
+        <v>580113701</v>
+      </c>
+      <c r="E71">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1118,12 +1622,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1131,115 +1635,232 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>46055</v>
       </c>
       <c r="B2">
+        <v>44109875</v>
+      </c>
+      <c r="C2">
+        <v>193229</v>
+      </c>
+      <c r="D2">
         <v>44303104</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>46062</v>
       </c>
       <c r="B3">
+        <v>24637511</v>
+      </c>
+      <c r="C3">
+        <v>73101</v>
+      </c>
+      <c r="D3">
         <v>24710612</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>46069</v>
       </c>
       <c r="B4">
+        <v>573734857</v>
+      </c>
+      <c r="C4">
+        <v>3603421</v>
+      </c>
+      <c r="D4">
         <v>577338278</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>463</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>46076</v>
       </c>
       <c r="B5">
+        <v>664132182</v>
+      </c>
+      <c r="C5">
+        <v>2647817</v>
+      </c>
+      <c r="D5">
         <v>666779999</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>663</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>46083</v>
       </c>
       <c r="B6">
+        <v>93745070</v>
+      </c>
+      <c r="C6">
+        <v>192787</v>
+      </c>
+      <c r="D6">
         <v>93937857</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>46090</v>
       </c>
       <c r="B7">
+        <v>1079662368</v>
+      </c>
+      <c r="C7">
+        <v>3515659</v>
+      </c>
+      <c r="D7">
         <v>1083178027</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>631</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>46097</v>
       </c>
       <c r="B8">
+        <v>955055968</v>
+      </c>
+      <c r="C8">
+        <v>2744430</v>
+      </c>
+      <c r="D8">
         <v>957800398</v>
       </c>
-      <c r="C8">
+      <c r="E8">
         <v>544</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>46104</v>
       </c>
       <c r="B9">
+        <v>1780982092</v>
+      </c>
+      <c r="C9">
+        <v>3800660</v>
+      </c>
+      <c r="D9">
         <v>1784782752</v>
       </c>
-      <c r="C9">
+      <c r="E9">
         <v>636</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>46111</v>
       </c>
       <c r="B10">
+        <v>3023435297</v>
+      </c>
+      <c r="C10">
+        <v>10787452</v>
+      </c>
+      <c r="D10">
         <v>3034222749</v>
       </c>
-      <c r="C10">
+      <c r="E10">
         <v>716</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1">
         <v>46118</v>
       </c>
       <c r="B11">
-        <v>137673542</v>
+        <v>1246212564</v>
       </c>
       <c r="C11">
-        <v>82</v>
+        <v>4215383</v>
+      </c>
+      <c r="D11">
+        <v>1250427947</v>
+      </c>
+      <c r="E11">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B12">
+        <v>1595054650</v>
+      </c>
+      <c r="C12">
+        <v>5713273</v>
+      </c>
+      <c r="D12">
+        <v>1600767923</v>
+      </c>
+      <c r="E12">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B13">
+        <v>3473700374</v>
+      </c>
+      <c r="C13">
+        <v>13160521</v>
+      </c>
+      <c r="D13">
+        <v>3486860895</v>
+      </c>
+      <c r="E13">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1">
+        <v>46139</v>
+      </c>
+      <c r="B14">
+        <v>742744555</v>
+      </c>
+      <c r="C14">
+        <v>2790054</v>
+      </c>
+      <c r="D14">
+        <v>745534609</v>
+      </c>
+      <c r="E14">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1249,12 +1870,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1262,27 +1883,517 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>46081</v>
       </c>
       <c r="B2">
+        <v>1313110878</v>
+      </c>
+      <c r="C2">
+        <v>6568396</v>
+      </c>
+      <c r="D2">
         <v>1319679274</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>1220</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>46112</v>
       </c>
       <c r="B3">
+        <v>7063569887</v>
+      </c>
+      <c r="C3">
+        <v>21478157</v>
+      </c>
+      <c r="D3">
         <v>7085048044</v>
       </c>
+      <c r="E3">
+        <v>2736</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1">
+        <v>46142</v>
+      </c>
+      <c r="B4">
+        <v>6920526598</v>
+      </c>
+      <c r="C4">
+        <v>25391234</v>
+      </c>
+      <c r="D4">
+        <v>6945917832</v>
+      </c>
+      <c r="E4">
+        <v>1408</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1">
+        <v>46122</v>
+      </c>
+      <c r="B2">
+        <v>116346489</v>
+      </c>
+      <c r="C2">
+        <v>289339</v>
+      </c>
+      <c r="D2">
+        <v>116635828</v>
+      </c>
+      <c r="E2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1">
+        <v>46123</v>
+      </c>
+      <c r="B3">
+        <v>160607016</v>
+      </c>
       <c r="C3">
-        <v>2736</v>
+        <v>686187</v>
+      </c>
+      <c r="D3">
+        <v>161293203</v>
+      </c>
+      <c r="E3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1">
+        <v>46124</v>
+      </c>
+      <c r="B4">
+        <v>475094565</v>
+      </c>
+      <c r="C4">
+        <v>1908297</v>
+      </c>
+      <c r="D4">
+        <v>477002862</v>
+      </c>
+      <c r="E4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B5">
+        <v>256361479</v>
+      </c>
+      <c r="C5">
+        <v>824687</v>
+      </c>
+      <c r="D5">
+        <v>257186166</v>
+      </c>
+      <c r="E5">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1">
+        <v>46126</v>
+      </c>
+      <c r="B6">
+        <v>277328285</v>
+      </c>
+      <c r="C6">
+        <v>875263</v>
+      </c>
+      <c r="D6">
+        <v>278203548</v>
+      </c>
+      <c r="E6">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1">
+        <v>46127</v>
+      </c>
+      <c r="B7">
+        <v>204982226</v>
+      </c>
+      <c r="C7">
+        <v>952185</v>
+      </c>
+      <c r="D7">
+        <v>205934411</v>
+      </c>
+      <c r="E7">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1">
+        <v>46128</v>
+      </c>
+      <c r="B8">
+        <v>984805312</v>
+      </c>
+      <c r="C8">
+        <v>3225513</v>
+      </c>
+      <c r="D8">
+        <v>988030825</v>
+      </c>
+      <c r="E8">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1">
+        <v>46129</v>
+      </c>
+      <c r="B9">
+        <v>481719807</v>
+      </c>
+      <c r="C9">
+        <v>1434059</v>
+      </c>
+      <c r="D9">
+        <v>483153866</v>
+      </c>
+      <c r="E9">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1">
+        <v>46130</v>
+      </c>
+      <c r="B10">
+        <v>984655867</v>
+      </c>
+      <c r="C10">
+        <v>4639910</v>
+      </c>
+      <c r="D10">
+        <v>989295777</v>
+      </c>
+      <c r="E10">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B11">
+        <v>540208877</v>
+      </c>
+      <c r="C11">
+        <v>2033591</v>
+      </c>
+      <c r="D11">
+        <v>542242468</v>
+      </c>
+      <c r="E11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B12">
+        <v>164639448</v>
+      </c>
+      <c r="C12">
+        <v>781460</v>
+      </c>
+      <c r="D12">
+        <v>165420908</v>
+      </c>
+      <c r="E12">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B13">
+        <v>578105107</v>
+      </c>
+      <c r="C13">
+        <v>2008594</v>
+      </c>
+      <c r="D13">
+        <v>580113701</v>
+      </c>
+      <c r="E13">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>4633458882</v>
+      </c>
+      <c r="C2">
+        <v>15884477</v>
+      </c>
+      <c r="D2">
+        <v>4649343359</v>
+      </c>
+      <c r="E2">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>511763645</v>
+      </c>
+      <c r="C3">
+        <v>1246354</v>
+      </c>
+      <c r="D3">
+        <v>513009999</v>
+      </c>
+      <c r="E3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>79631938</v>
+      </c>
+      <c r="C4">
+        <v>2528254</v>
+      </c>
+      <c r="D4">
+        <v>82160192</v>
+      </c>
+      <c r="E4">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>4260456671</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>4260456671</v>
+      </c>
+      <c r="E2">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>807020429</v>
+      </c>
+      <c r="C3">
+        <v>19659085</v>
+      </c>
+      <c r="D3">
+        <v>826679514</v>
+      </c>
+      <c r="E3">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>157377365</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>157377365</v>
+      </c>
+      <c r="E4">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(v2.8.0): add project analysis report and assessment documents (#1822)
- Add comprehensive v2.8.0 project analysis report (docs/report/)
- Add project analysis guide with workflow and tool instructions
- Add v2.8.0 version-specific analysis report (docs/governance/reports/)
- Update Minimax usage analysis with latest CSV data (04-24)
- Update trend chart scripts and generated charts
- Update 项目分析报告.md with latest data through 04-22

Key findings:
- v2.8.0: 81 PRs in 2 days, distributed features (GTID/semi-sync/read-write split)
- Minimax: 4.37B tokens/day (last 2 weeks), +44.3% vs prior 2 weeks
- TPC-H SF=1: 22/22 queries pass, total ~4.2s (v2.7.0)
- Sysbench OLTP: 55K TPS point select, 22K TPS insert
- Documentation PRs at 31.7% - project entering maturity phase

Co-authored-by: Li Ying <openheart@gaoyuanyiyao.com>
</commit_message>
<xml_diff>
--- a/scripts/usage/minimax_usage_summary.xlsx
+++ b/scripts/usage/minimax_usage_summary.xlsx
@@ -10,13 +10,22 @@
     <sheet name="每日汇总" sheetId="1" r:id="rId1"/>
     <sheet name="每周汇总" sheetId="2" r:id="rId2"/>
     <sheet name="每月汇总" sheetId="3" r:id="rId3"/>
+    <sheet name="最近2周" sheetId="4" r:id="rId4"/>
+    <sheet name="模型分布" sheetId="5" r:id="rId5"/>
+    <sheet name="接口分布" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="17">
+  <si>
+    <t>输入消费数</t>
+  </si>
+  <si>
+    <t>输出消费数</t>
+  </si>
   <si>
     <t>总消费数</t>
   </si>
@@ -25,6 +34,42 @@
   </si>
   <si>
     <t>日期</t>
+  </si>
+  <si>
+    <t>消费模型</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.7-highspeed</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.1</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.7</t>
+  </si>
+  <si>
+    <t>coding-plan-search</t>
+  </si>
+  <si>
+    <t>subscribe</t>
+  </si>
+  <si>
+    <t>消费接口</t>
+  </si>
+  <si>
+    <t>cache-read(Text API)</t>
+  </si>
+  <si>
+    <t>chatcompletion-v2(Text API)</t>
+  </si>
+  <si>
+    <t>cache-create(Text API)</t>
+  </si>
+  <si>
+    <t>code_plan_resource_package</t>
+  </si>
+  <si>
+    <t>code_plan_purchase</t>
   </si>
 </sst>
 </file>
@@ -360,12 +405,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -373,742 +418,1201 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>46055</v>
       </c>
       <c r="B2">
+        <v>44109875</v>
+      </c>
+      <c r="C2">
+        <v>193229</v>
+      </c>
+      <c r="D2">
         <v>44303104</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>46056</v>
       </c>
       <c r="B3">
+        <v>24346019</v>
+      </c>
+      <c r="C3">
+        <v>69189</v>
+      </c>
+      <c r="D3">
         <v>24415208</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>46058</v>
       </c>
       <c r="B4">
+        <v>68473</v>
+      </c>
+      <c r="C4">
+        <v>723</v>
+      </c>
+      <c r="D4">
         <v>69196</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>46062</v>
       </c>
       <c r="B5">
+        <v>223019</v>
+      </c>
+      <c r="C5">
+        <v>3189</v>
+      </c>
+      <c r="D5">
         <v>226208</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>46064</v>
       </c>
       <c r="B6">
+        <v>1625031</v>
+      </c>
+      <c r="C6">
+        <v>50080</v>
+      </c>
+      <c r="D6">
         <v>1675111</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>46065</v>
       </c>
       <c r="B7">
+        <v>10098026</v>
+      </c>
+      <c r="C7">
+        <v>80296</v>
+      </c>
+      <c r="D7">
         <v>10178322</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>46066</v>
       </c>
       <c r="B8">
+        <v>195262132</v>
+      </c>
+      <c r="C8">
+        <v>1014368</v>
+      </c>
+      <c r="D8">
         <v>196276500</v>
       </c>
-      <c r="C8">
+      <c r="E8">
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>46067</v>
       </c>
       <c r="B9">
+        <v>118553679</v>
+      </c>
+      <c r="C9">
+        <v>540118</v>
+      </c>
+      <c r="D9">
         <v>119093797</v>
       </c>
-      <c r="C9">
+      <c r="E9">
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>46068</v>
       </c>
       <c r="B10">
+        <v>107894789</v>
+      </c>
+      <c r="C10">
+        <v>740115</v>
+      </c>
+      <c r="D10">
         <v>108634904</v>
       </c>
-      <c r="C10">
+      <c r="E10">
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1">
         <v>46069</v>
       </c>
       <c r="B11">
+        <v>140301200</v>
+      </c>
+      <c r="C11">
+        <v>1178444</v>
+      </c>
+      <c r="D11">
         <v>141479644</v>
       </c>
-      <c r="C11">
+      <c r="E11">
         <v>144</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:5">
       <c r="A12" s="1">
         <v>46070</v>
       </c>
       <c r="B12">
+        <v>170014054</v>
+      </c>
+      <c r="C12">
+        <v>606139</v>
+      </c>
+      <c r="D12">
         <v>170620193</v>
       </c>
-      <c r="C12">
+      <c r="E12">
         <v>144</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:5">
       <c r="A13" s="1">
         <v>46071</v>
       </c>
       <c r="B13">
+        <v>121481164</v>
+      </c>
+      <c r="C13">
+        <v>452181</v>
+      </c>
+      <c r="D13">
         <v>121933345</v>
       </c>
-      <c r="C13">
+      <c r="E13">
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:5">
       <c r="A14" s="1">
         <v>46072</v>
       </c>
       <c r="B14">
+        <v>39782200</v>
+      </c>
+      <c r="C14">
+        <v>294745</v>
+      </c>
+      <c r="D14">
         <v>40076945</v>
       </c>
-      <c r="C14">
+      <c r="E14">
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:5">
       <c r="A15" s="1">
         <v>46073</v>
       </c>
       <c r="B15">
+        <v>259713471</v>
+      </c>
+      <c r="C15">
+        <v>1000667</v>
+      </c>
+      <c r="D15">
         <v>260714138</v>
       </c>
-      <c r="C15">
+      <c r="E15">
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:5">
       <c r="A16" s="1">
         <v>46074</v>
       </c>
       <c r="B16">
+        <v>66491505</v>
+      </c>
+      <c r="C16">
+        <v>247164</v>
+      </c>
+      <c r="D16">
         <v>66738669</v>
       </c>
-      <c r="C16">
+      <c r="E16">
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:5">
       <c r="A17" s="1">
         <v>46075</v>
       </c>
       <c r="B17">
+        <v>5513297</v>
+      </c>
+      <c r="C17">
+        <v>42902</v>
+      </c>
+      <c r="D17">
         <v>5556199</v>
       </c>
-      <c r="C17">
+      <c r="E17">
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:5">
       <c r="A18" s="1">
         <v>46076</v>
       </c>
       <c r="B18">
+        <v>1136491</v>
+      </c>
+      <c r="C18">
+        <v>4019</v>
+      </c>
+      <c r="D18">
         <v>1140510</v>
       </c>
-      <c r="C18">
+      <c r="E18">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:5">
       <c r="A19" s="1">
         <v>46077</v>
       </c>
       <c r="B19">
+        <v>2606410</v>
+      </c>
+      <c r="C19">
+        <v>26537</v>
+      </c>
+      <c r="D19">
         <v>2632947</v>
       </c>
-      <c r="C19">
+      <c r="E19">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:5">
       <c r="A20" s="1">
         <v>46081</v>
       </c>
       <c r="B20">
+        <v>3890043</v>
+      </c>
+      <c r="C20">
+        <v>24291</v>
+      </c>
+      <c r="D20">
         <v>3914334</v>
       </c>
-      <c r="C20">
+      <c r="E20">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:5">
       <c r="A21" s="1">
         <v>46082</v>
       </c>
       <c r="B21">
+        <v>76442533</v>
+      </c>
+      <c r="C21">
+        <v>111170</v>
+      </c>
+      <c r="D21">
         <v>76553703</v>
       </c>
-      <c r="C21">
+      <c r="E21">
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:5">
       <c r="A22" s="1">
         <v>46083</v>
       </c>
       <c r="B22">
+        <v>10806084</v>
+      </c>
+      <c r="C22">
+        <v>30789</v>
+      </c>
+      <c r="D22">
         <v>10836873</v>
       </c>
-      <c r="C22">
+      <c r="E22">
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:5">
       <c r="A23" s="1">
         <v>46084</v>
       </c>
       <c r="B23">
+        <v>260321813</v>
+      </c>
+      <c r="C23">
+        <v>949069</v>
+      </c>
+      <c r="D23">
         <v>261270882</v>
       </c>
-      <c r="C23">
+      <c r="E23">
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:5">
       <c r="A24" s="1">
         <v>46085</v>
       </c>
       <c r="B24">
+        <v>57609431</v>
+      </c>
+      <c r="C24">
+        <v>169857</v>
+      </c>
+      <c r="D24">
         <v>57779288</v>
       </c>
-      <c r="C24">
+      <c r="E24">
         <v>88</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:5">
       <c r="A25" s="1">
         <v>46086</v>
       </c>
       <c r="B25">
+        <v>432659759</v>
+      </c>
+      <c r="C25">
+        <v>1367934</v>
+      </c>
+      <c r="D25">
         <v>434027693</v>
       </c>
-      <c r="C25">
+      <c r="E25">
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:5">
       <c r="A26" s="1">
         <v>46087</v>
       </c>
       <c r="B26">
+        <v>69824048</v>
+      </c>
+      <c r="C26">
+        <v>126022</v>
+      </c>
+      <c r="D26">
         <v>69950070</v>
       </c>
-      <c r="C26">
+      <c r="E26">
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:5">
       <c r="A27" s="1">
         <v>46088</v>
       </c>
       <c r="B27">
+        <v>123888083</v>
+      </c>
+      <c r="C27">
+        <v>526914</v>
+      </c>
+      <c r="D27">
         <v>124414997</v>
       </c>
-      <c r="C27">
+      <c r="E27">
         <v>96</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:5">
       <c r="A28" s="1">
         <v>46089</v>
       </c>
       <c r="B28">
+        <v>94927345</v>
+      </c>
+      <c r="C28">
+        <v>206477</v>
+      </c>
+      <c r="D28">
         <v>95133822</v>
       </c>
-      <c r="C28">
+      <c r="E28">
         <v>104</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:5">
       <c r="A29" s="1">
         <v>46090</v>
       </c>
       <c r="B29">
+        <v>40431889</v>
+      </c>
+      <c r="C29">
+        <v>169386</v>
+      </c>
+      <c r="D29">
         <v>40601275</v>
       </c>
-      <c r="C29">
+      <c r="E29">
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:5">
       <c r="A30" s="1">
         <v>46091</v>
       </c>
       <c r="B30">
+        <v>17773567</v>
+      </c>
+      <c r="C30">
+        <v>99491</v>
+      </c>
+      <c r="D30">
         <v>17873058</v>
       </c>
-      <c r="C30">
+      <c r="E30">
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:5">
       <c r="A31" s="1">
         <v>46092</v>
       </c>
       <c r="B31">
+        <v>217635219</v>
+      </c>
+      <c r="C31">
+        <v>736629</v>
+      </c>
+      <c r="D31">
         <v>218371848</v>
       </c>
-      <c r="C31">
+      <c r="E31">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:5">
       <c r="A32" s="1">
         <v>46093</v>
       </c>
       <c r="B32">
+        <v>65692490</v>
+      </c>
+      <c r="C32">
+        <v>208372</v>
+      </c>
+      <c r="D32">
         <v>65900862</v>
       </c>
-      <c r="C32">
+      <c r="E32">
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:5">
       <c r="A33" s="1">
         <v>46094</v>
       </c>
       <c r="B33">
+        <v>150670082</v>
+      </c>
+      <c r="C33">
+        <v>508790</v>
+      </c>
+      <c r="D33">
         <v>151178872</v>
       </c>
-      <c r="C33">
+      <c r="E33">
         <v>87</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:5">
       <c r="A34" s="1">
         <v>46095</v>
       </c>
       <c r="B34">
+        <v>131208124</v>
+      </c>
+      <c r="C34">
+        <v>318055</v>
+      </c>
+      <c r="D34">
         <v>131526179</v>
       </c>
-      <c r="C34">
+      <c r="E34">
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:5">
       <c r="A35" s="1">
         <v>46096</v>
       </c>
       <c r="B35">
+        <v>229056688</v>
+      </c>
+      <c r="C35">
+        <v>539232</v>
+      </c>
+      <c r="D35">
         <v>229595920</v>
       </c>
-      <c r="C35">
+      <c r="E35">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:5">
       <c r="A36" s="1">
         <v>46097</v>
       </c>
       <c r="B36">
+        <v>143019798</v>
+      </c>
+      <c r="C36">
+        <v>333861</v>
+      </c>
+      <c r="D36">
         <v>143353659</v>
       </c>
-      <c r="C36">
+      <c r="E36">
         <v>93</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:5">
       <c r="A37" s="1">
         <v>46098</v>
       </c>
       <c r="B37">
+        <v>11928233</v>
+      </c>
+      <c r="C37">
+        <v>51737</v>
+      </c>
+      <c r="D37">
         <v>11979970</v>
       </c>
-      <c r="C37">
+      <c r="E37">
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:5">
       <c r="A38" s="1">
         <v>46099</v>
       </c>
       <c r="B38">
+        <v>399975698</v>
+      </c>
+      <c r="C38">
+        <v>772414</v>
+      </c>
+      <c r="D38">
         <v>400748112</v>
       </c>
-      <c r="C38">
+      <c r="E38">
         <v>96</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:5">
       <c r="A39" s="1">
         <v>46100</v>
       </c>
       <c r="B39">
+        <v>609350469</v>
+      </c>
+      <c r="C39">
+        <v>1236187</v>
+      </c>
+      <c r="D39">
         <v>610586656</v>
       </c>
-      <c r="C39">
+      <c r="E39">
         <v>106</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:5">
       <c r="A40" s="1">
         <v>46101</v>
       </c>
       <c r="B40">
+        <v>256702111</v>
+      </c>
+      <c r="C40">
+        <v>469772</v>
+      </c>
+      <c r="D40">
         <v>257171883</v>
       </c>
-      <c r="C40">
+      <c r="E40">
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:5">
       <c r="A41" s="1">
         <v>46102</v>
       </c>
       <c r="B41">
+        <v>395205934</v>
+      </c>
+      <c r="C41">
+        <v>970120</v>
+      </c>
+      <c r="D41">
         <v>396176054</v>
       </c>
-      <c r="C41">
+      <c r="E41">
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:5">
       <c r="A42" s="1">
         <v>46103</v>
       </c>
       <c r="B42">
+        <v>24127943</v>
+      </c>
+      <c r="C42">
+        <v>86128</v>
+      </c>
+      <c r="D42">
         <v>24214071</v>
       </c>
-      <c r="C42">
+      <c r="E42">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:5">
       <c r="A43" s="1">
         <v>46104</v>
       </c>
       <c r="B43">
+        <v>83691704</v>
+      </c>
+      <c r="C43">
+        <v>214302</v>
+      </c>
+      <c r="D43">
         <v>83906006</v>
       </c>
-      <c r="C43">
+      <c r="E43">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:5">
       <c r="A44" s="1">
         <v>46105</v>
       </c>
       <c r="B44">
+        <v>69644470</v>
+      </c>
+      <c r="C44">
+        <v>207355</v>
+      </c>
+      <c r="D44">
         <v>69851825</v>
       </c>
-      <c r="C44">
+      <c r="E44">
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:5">
       <c r="A45" s="1">
         <v>46106</v>
       </c>
       <c r="B45">
+        <v>61827053</v>
+      </c>
+      <c r="C45">
+        <v>125764</v>
+      </c>
+      <c r="D45">
         <v>61952817</v>
       </c>
-      <c r="C45">
+      <c r="E45">
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:5">
       <c r="A46" s="1">
         <v>46107</v>
       </c>
       <c r="B46">
+        <v>801621176</v>
+      </c>
+      <c r="C46">
+        <v>3000001</v>
+      </c>
+      <c r="D46">
         <v>804621177</v>
       </c>
-      <c r="C46">
+      <c r="E46">
         <v>121</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:5">
       <c r="A47" s="1">
         <v>46108</v>
       </c>
       <c r="B47">
+        <v>410302751</v>
+      </c>
+      <c r="C47">
+        <v>1260959</v>
+      </c>
+      <c r="D47">
         <v>411563710</v>
       </c>
-      <c r="C47">
+      <c r="E47">
         <v>79</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:5">
       <c r="A48" s="1">
         <v>46109</v>
       </c>
       <c r="B48">
+        <v>669961980</v>
+      </c>
+      <c r="C48">
+        <v>2390124</v>
+      </c>
+      <c r="D48">
         <v>672352104</v>
       </c>
-      <c r="C48">
+      <c r="E48">
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:5">
       <c r="A49" s="1">
         <v>46110</v>
       </c>
       <c r="B49">
+        <v>781214642</v>
+      </c>
+      <c r="C49">
+        <v>2860496</v>
+      </c>
+      <c r="D49">
         <v>784075138</v>
       </c>
-      <c r="C49">
+      <c r="E49">
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:5">
       <c r="A50" s="1">
         <v>46111</v>
       </c>
       <c r="B50">
+        <v>228863225</v>
+      </c>
+      <c r="C50">
+        <v>942753</v>
+      </c>
+      <c r="D50">
         <v>229805978</v>
       </c>
-      <c r="C50">
+      <c r="E50">
         <v>80</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:5">
       <c r="A51" s="1">
         <v>46112</v>
       </c>
       <c r="B51">
+        <v>137185545</v>
+      </c>
+      <c r="C51">
+        <v>487997</v>
+      </c>
+      <c r="D51">
         <v>137673542</v>
       </c>
-      <c r="C51">
+      <c r="E51">
         <v>82</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:5">
       <c r="A52" s="1">
         <v>46113</v>
       </c>
       <c r="B52">
+        <v>315751692</v>
+      </c>
+      <c r="C52">
+        <v>1016666</v>
+      </c>
+      <c r="D52">
         <v>316768358</v>
       </c>
-      <c r="C52">
+      <c r="E52">
         <v>87</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:5">
       <c r="A53" s="1">
         <v>46114</v>
       </c>
       <c r="B53">
+        <v>455846463</v>
+      </c>
+      <c r="C53">
+        <v>1163341</v>
+      </c>
+      <c r="D53">
         <v>457009804</v>
       </c>
-      <c r="C53">
+      <c r="E53">
         <v>80</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:5">
       <c r="A54" s="1">
         <v>46115</v>
       </c>
       <c r="B54">
+        <v>173451910</v>
+      </c>
+      <c r="C54">
+        <v>867510</v>
+      </c>
+      <c r="D54">
         <v>174319420</v>
       </c>
-      <c r="C54">
+      <c r="E54">
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:5">
       <c r="A55" s="1">
         <v>46116</v>
       </c>
       <c r="B55">
+        <v>163888833</v>
+      </c>
+      <c r="C55">
+        <v>679765</v>
+      </c>
+      <c r="D55">
         <v>164568598</v>
       </c>
-      <c r="C55">
+      <c r="E55">
         <v>93</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:5">
       <c r="A56" s="1">
         <v>46117</v>
       </c>
       <c r="B56">
+        <v>88121</v>
+      </c>
+      <c r="C56">
+        <v>104</v>
+      </c>
+      <c r="D56">
         <v>88225</v>
       </c>
-      <c r="C56">
+      <c r="E56">
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:5">
       <c r="A57" s="1">
         <v>46119</v>
       </c>
       <c r="B57">
+        <v>52904173</v>
+      </c>
+      <c r="C57">
+        <v>607681</v>
+      </c>
+      <c r="D57">
         <v>53511854</v>
       </c>
-      <c r="C57">
+      <c r="E57">
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:5">
       <c r="A58" s="1">
         <v>46120</v>
       </c>
       <c r="B58">
+        <v>224034425</v>
+      </c>
+      <c r="C58">
+        <v>522473</v>
+      </c>
+      <c r="D58">
         <v>224556898</v>
       </c>
-      <c r="C58">
+      <c r="E58">
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:5">
       <c r="A59" s="1">
         <v>46121</v>
       </c>
       <c r="B59">
+        <v>309706503</v>
+      </c>
+      <c r="C59">
+        <v>874609</v>
+      </c>
+      <c r="D59">
         <v>310581112</v>
       </c>
-      <c r="C59">
+      <c r="E59">
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:5">
       <c r="A60" s="1">
         <v>46122</v>
       </c>
       <c r="B60">
+        <v>116346489</v>
+      </c>
+      <c r="C60">
+        <v>289339</v>
+      </c>
+      <c r="D60">
         <v>116635828</v>
       </c>
-      <c r="C60">
+      <c r="E60">
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:5">
       <c r="A61" s="1">
         <v>46123</v>
       </c>
       <c r="B61">
+        <v>160607016</v>
+      </c>
+      <c r="C61">
+        <v>686187</v>
+      </c>
+      <c r="D61">
         <v>161293203</v>
       </c>
-      <c r="C61">
+      <c r="E61">
         <v>54</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:5">
       <c r="A62" s="1">
         <v>46124</v>
       </c>
       <c r="B62">
+        <v>475094565</v>
+      </c>
+      <c r="C62">
+        <v>1908297</v>
+      </c>
+      <c r="D62">
         <v>477002862</v>
       </c>
-      <c r="C62">
+      <c r="E62">
         <v>82</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:5">
       <c r="A63" s="1">
         <v>46125</v>
       </c>
       <c r="B63">
+        <v>256361479</v>
+      </c>
+      <c r="C63">
+        <v>824687</v>
+      </c>
+      <c r="D63">
         <v>257186166</v>
       </c>
-      <c r="C63">
+      <c r="E63">
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:5">
       <c r="A64" s="1">
         <v>46126</v>
       </c>
       <c r="B64">
+        <v>277328285</v>
+      </c>
+      <c r="C64">
+        <v>875263</v>
+      </c>
+      <c r="D64">
         <v>278203548</v>
       </c>
-      <c r="C64">
+      <c r="E64">
         <v>102</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:5">
       <c r="A65" s="1">
         <v>46127</v>
       </c>
       <c r="B65">
+        <v>204982226</v>
+      </c>
+      <c r="C65">
+        <v>952185</v>
+      </c>
+      <c r="D65">
         <v>205934411</v>
       </c>
-      <c r="C65">
+      <c r="E65">
         <v>69</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:5">
       <c r="A66" s="1">
         <v>46128</v>
       </c>
       <c r="B66">
+        <v>984805312</v>
+      </c>
+      <c r="C66">
+        <v>3225513</v>
+      </c>
+      <c r="D66">
         <v>988030825</v>
       </c>
-      <c r="C66">
+      <c r="E66">
         <v>93</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:5">
       <c r="A67" s="1">
         <v>46129</v>
       </c>
       <c r="B67">
+        <v>481719807</v>
+      </c>
+      <c r="C67">
+        <v>1434059</v>
+      </c>
+      <c r="D67">
         <v>483153866</v>
       </c>
-      <c r="C67">
+      <c r="E67">
         <v>104</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:5">
       <c r="A68" s="1">
         <v>46130</v>
       </c>
       <c r="B68">
+        <v>984655867</v>
+      </c>
+      <c r="C68">
+        <v>4639910</v>
+      </c>
+      <c r="D68">
         <v>989295777</v>
       </c>
-      <c r="C68">
+      <c r="E68">
         <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B69">
+        <v>540208877</v>
+      </c>
+      <c r="C69">
+        <v>2033591</v>
+      </c>
+      <c r="D69">
+        <v>542242468</v>
+      </c>
+      <c r="E69">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B70">
+        <v>164639448</v>
+      </c>
+      <c r="C70">
+        <v>781460</v>
+      </c>
+      <c r="D70">
+        <v>165420908</v>
+      </c>
+      <c r="E70">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B71">
+        <v>578105107</v>
+      </c>
+      <c r="C71">
+        <v>2008594</v>
+      </c>
+      <c r="D71">
+        <v>580113701</v>
+      </c>
+      <c r="E71">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1118,12 +1622,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1131,115 +1635,232 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>46055</v>
       </c>
       <c r="B2">
+        <v>44109875</v>
+      </c>
+      <c r="C2">
+        <v>193229</v>
+      </c>
+      <c r="D2">
         <v>44303104</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>46062</v>
       </c>
       <c r="B3">
+        <v>24637511</v>
+      </c>
+      <c r="C3">
+        <v>73101</v>
+      </c>
+      <c r="D3">
         <v>24710612</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>46069</v>
       </c>
       <c r="B4">
+        <v>573734857</v>
+      </c>
+      <c r="C4">
+        <v>3603421</v>
+      </c>
+      <c r="D4">
         <v>577338278</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>463</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>46076</v>
       </c>
       <c r="B5">
+        <v>664132182</v>
+      </c>
+      <c r="C5">
+        <v>2647817</v>
+      </c>
+      <c r="D5">
         <v>666779999</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>663</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>46083</v>
       </c>
       <c r="B6">
+        <v>93745070</v>
+      </c>
+      <c r="C6">
+        <v>192787</v>
+      </c>
+      <c r="D6">
         <v>93937857</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>46090</v>
       </c>
       <c r="B7">
+        <v>1079662368</v>
+      </c>
+      <c r="C7">
+        <v>3515659</v>
+      </c>
+      <c r="D7">
         <v>1083178027</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>631</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>46097</v>
       </c>
       <c r="B8">
+        <v>955055968</v>
+      </c>
+      <c r="C8">
+        <v>2744430</v>
+      </c>
+      <c r="D8">
         <v>957800398</v>
       </c>
-      <c r="C8">
+      <c r="E8">
         <v>544</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>46104</v>
       </c>
       <c r="B9">
+        <v>1780982092</v>
+      </c>
+      <c r="C9">
+        <v>3800660</v>
+      </c>
+      <c r="D9">
         <v>1784782752</v>
       </c>
-      <c r="C9">
+      <c r="E9">
         <v>636</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>46111</v>
       </c>
       <c r="B10">
+        <v>3023435297</v>
+      </c>
+      <c r="C10">
+        <v>10787452</v>
+      </c>
+      <c r="D10">
         <v>3034222749</v>
       </c>
-      <c r="C10">
+      <c r="E10">
         <v>716</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1">
         <v>46118</v>
       </c>
       <c r="B11">
-        <v>137673542</v>
+        <v>1246212564</v>
       </c>
       <c r="C11">
-        <v>82</v>
+        <v>4215383</v>
+      </c>
+      <c r="D11">
+        <v>1250427947</v>
+      </c>
+      <c r="E11">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B12">
+        <v>1595054650</v>
+      </c>
+      <c r="C12">
+        <v>5713273</v>
+      </c>
+      <c r="D12">
+        <v>1600767923</v>
+      </c>
+      <c r="E12">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B13">
+        <v>3473700374</v>
+      </c>
+      <c r="C13">
+        <v>13160521</v>
+      </c>
+      <c r="D13">
+        <v>3486860895</v>
+      </c>
+      <c r="E13">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1">
+        <v>46139</v>
+      </c>
+      <c r="B14">
+        <v>742744555</v>
+      </c>
+      <c r="C14">
+        <v>2790054</v>
+      </c>
+      <c r="D14">
+        <v>745534609</v>
+      </c>
+      <c r="E14">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1249,12 +1870,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1262,27 +1883,517 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="1">
         <v>46081</v>
       </c>
       <c r="B2">
+        <v>1313110878</v>
+      </c>
+      <c r="C2">
+        <v>6568396</v>
+      </c>
+      <c r="D2">
         <v>1319679274</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>1220</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>46112</v>
       </c>
       <c r="B3">
+        <v>7063569887</v>
+      </c>
+      <c r="C3">
+        <v>21478157</v>
+      </c>
+      <c r="D3">
         <v>7085048044</v>
       </c>
+      <c r="E3">
+        <v>2736</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1">
+        <v>46142</v>
+      </c>
+      <c r="B4">
+        <v>6920526598</v>
+      </c>
+      <c r="C4">
+        <v>25391234</v>
+      </c>
+      <c r="D4">
+        <v>6945917832</v>
+      </c>
+      <c r="E4">
+        <v>1408</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1">
+        <v>46122</v>
+      </c>
+      <c r="B2">
+        <v>116346489</v>
+      </c>
+      <c r="C2">
+        <v>289339</v>
+      </c>
+      <c r="D2">
+        <v>116635828</v>
+      </c>
+      <c r="E2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1">
+        <v>46123</v>
+      </c>
+      <c r="B3">
+        <v>160607016</v>
+      </c>
       <c r="C3">
-        <v>2736</v>
+        <v>686187</v>
+      </c>
+      <c r="D3">
+        <v>161293203</v>
+      </c>
+      <c r="E3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1">
+        <v>46124</v>
+      </c>
+      <c r="B4">
+        <v>475094565</v>
+      </c>
+      <c r="C4">
+        <v>1908297</v>
+      </c>
+      <c r="D4">
+        <v>477002862</v>
+      </c>
+      <c r="E4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B5">
+        <v>256361479</v>
+      </c>
+      <c r="C5">
+        <v>824687</v>
+      </c>
+      <c r="D5">
+        <v>257186166</v>
+      </c>
+      <c r="E5">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1">
+        <v>46126</v>
+      </c>
+      <c r="B6">
+        <v>277328285</v>
+      </c>
+      <c r="C6">
+        <v>875263</v>
+      </c>
+      <c r="D6">
+        <v>278203548</v>
+      </c>
+      <c r="E6">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1">
+        <v>46127</v>
+      </c>
+      <c r="B7">
+        <v>204982226</v>
+      </c>
+      <c r="C7">
+        <v>952185</v>
+      </c>
+      <c r="D7">
+        <v>205934411</v>
+      </c>
+      <c r="E7">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1">
+        <v>46128</v>
+      </c>
+      <c r="B8">
+        <v>984805312</v>
+      </c>
+      <c r="C8">
+        <v>3225513</v>
+      </c>
+      <c r="D8">
+        <v>988030825</v>
+      </c>
+      <c r="E8">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1">
+        <v>46129</v>
+      </c>
+      <c r="B9">
+        <v>481719807</v>
+      </c>
+      <c r="C9">
+        <v>1434059</v>
+      </c>
+      <c r="D9">
+        <v>483153866</v>
+      </c>
+      <c r="E9">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1">
+        <v>46130</v>
+      </c>
+      <c r="B10">
+        <v>984655867</v>
+      </c>
+      <c r="C10">
+        <v>4639910</v>
+      </c>
+      <c r="D10">
+        <v>989295777</v>
+      </c>
+      <c r="E10">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B11">
+        <v>540208877</v>
+      </c>
+      <c r="C11">
+        <v>2033591</v>
+      </c>
+      <c r="D11">
+        <v>542242468</v>
+      </c>
+      <c r="E11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B12">
+        <v>164639448</v>
+      </c>
+      <c r="C12">
+        <v>781460</v>
+      </c>
+      <c r="D12">
+        <v>165420908</v>
+      </c>
+      <c r="E12">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B13">
+        <v>578105107</v>
+      </c>
+      <c r="C13">
+        <v>2008594</v>
+      </c>
+      <c r="D13">
+        <v>580113701</v>
+      </c>
+      <c r="E13">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>4633458882</v>
+      </c>
+      <c r="C2">
+        <v>15884477</v>
+      </c>
+      <c r="D2">
+        <v>4649343359</v>
+      </c>
+      <c r="E2">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>511763645</v>
+      </c>
+      <c r="C3">
+        <v>1246354</v>
+      </c>
+      <c r="D3">
+        <v>513009999</v>
+      </c>
+      <c r="E3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>79631938</v>
+      </c>
+      <c r="C4">
+        <v>2528254</v>
+      </c>
+      <c r="D4">
+        <v>82160192</v>
+      </c>
+      <c r="E4">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>4260456671</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>4260456671</v>
+      </c>
+      <c r="E2">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>807020429</v>
+      </c>
+      <c r="C3">
+        <v>19659085</v>
+      </c>
+      <c r="D3">
+        <v>826679514</v>
+      </c>
+      <c r="E3">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>157377365</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>157377365</v>
+      </c>
+      <c r="E4">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>